<commit_message>
feat: preserve Excel data during template migration
</commit_message>
<xml_diff>
--- a/gd/excel/Item.xlsx
+++ b/gd/excel/Item.xlsx
@@ -17,19 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="微软雅黑"/>
@@ -47,8 +41,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001B4332"/>
+        <bgColor rgb="001B4332"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C9A227"/>
         <bgColor rgb="00C9A227"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0040916C"/>
+        <bgColor rgb="0040916C"/>
       </patternFill>
     </fill>
     <fill>
@@ -57,20 +63,8 @@
         <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B4332"/>
-        <bgColor rgb="001B4332"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0040916C"/>
-        <bgColor rgb="0040916C"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -83,27 +77,6 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -130,22 +103,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -570,7 +542,7 @@
       <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Name
-string[i18n]</t>
+string</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -582,26 +554,26 @@
       <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Rarity
-enum[common,rare,epic]</t>
+ItemRarity</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
           <t>ItemTypeId
-int32[ref:ItemType.Id]</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
+int32</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>DropRange
-Droprange</t>
+ItemDropRange</t>
         </is>
       </c>
       <c r="G1" s="6" t="n"/>
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Tags
-array&lt;int32&gt;</t>
+vector&lt;int32&gt;</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
@@ -612,25 +584,13 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="7" t="n"/>
-      <c r="B2" s="7" t="n"/>
-      <c r="C2" s="7" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Min
-int32</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Max
-int32</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Min
+</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -820,15 +780,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="I1:I2"/>
+  <mergeCells count="2">
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:I1000">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>